<commit_message>
feat: deepen audit engine with graph export and SS008
</commit_message>
<xml_diff>
--- a/fixtures/bad_model.xlsx
+++ b/fixtures/bad_model.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Input</t>
   </si>
@@ -47,6 +47,9 @@
     <t>Inflated</t>
   </si>
   <si>
+    <t>Multiplier</t>
+  </si>
+  <si>
     <t>Rent</t>
   </si>
   <si>
@@ -78,6 +81,9 @@
   </si>
   <si>
     <t>Broken lookup</t>
+  </si>
+  <si>
+    <t>External link</t>
   </si>
   <si>
     <t>Tax model</t>
@@ -468,10 +474,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -481,64 +487,70 @@
       <c r="C1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>100</v>
       </c>
       <c r="C2">
-        <f>B2*$C$2</f>
+        <f>B2*$D$2</f>
         <v>110.00000000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>120</v>
       </c>
       <c r="C3">
-        <f>B3*$C$2</f>
+        <f>B3*$D$2</f>
         <v>132.0</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>130</v>
       </c>
       <c r="C4">
-        <f>B4*$C$2</f>
+        <f>B4*$D$2</f>
         <v>143.0</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>140</v>
       </c>
       <c r="C5">
-        <f>B5*$C$2</f>
+        <f>B5*$D$2</f>
         <v>154.0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1">
+    <row r="6" spans="1:4" hidden="1">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>150</v>
       </c>
       <c r="C6">
-        <f>B7*$C$2</f>
+        <f>B7*$D$2</f>
         <v>0</v>
       </c>
     </row>
@@ -549,12 +561,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -562,7 +574,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <f>Inputs!B2*1.05</f>
@@ -571,7 +583,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <f>SUM(Opex!C2:C6)</f>
@@ -580,7 +592,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" t="e">
         <f>#REF!</f>
@@ -589,7 +601,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <f>TODAY()</f>
@@ -598,11 +610,20 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" t="e">
         <f>NA()</f>
         <v>#N/A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7">
+        <f>'[Book2.xlsx]Sheet1'!A1</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -617,15 +638,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3">
         <f>D3*0.1</f>

</xml_diff>

<commit_message>
feat: config files and two additional audit rules
</commit_message>
<xml_diff>
--- a/fixtures/bad_model.xlsx
+++ b/fixtures/bad_model.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>Input</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>External link</t>
+  </si>
+  <si>
+    <t>Whole column</t>
+  </si>
+  <si>
+    <t>Uncached formula</t>
   </si>
   <si>
     <t>Tax model</t>
@@ -561,7 +567,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -624,6 +630,23 @@
       <c r="B7">
         <f>'[Book2.xlsx]Sheet1'!A1</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8">
+        <f>SUM(Opex!C:C)</f>
+        <v>660</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <f>1+1</f>
       </c>
     </row>
   </sheetData>
@@ -638,15 +661,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3">
         <f>D3*0.1</f>

</xml_diff>

<commit_message>
feat: support named, dynamic, structured, and external slice dependencies
</commit_message>
<xml_diff>
--- a/fixtures/bad_model.xlsx
+++ b/fixtures/bad_model.xlsx
@@ -13,12 +13,15 @@
     <sheet name="Tax" sheetId="4" r:id="rId4"/>
     <sheet name="Scratch" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="RevenueInput">Inputs!$B$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t>Input</t>
   </si>
@@ -90,6 +93,21 @@
   </si>
   <si>
     <t>Uncached formula</t>
+  </si>
+  <si>
+    <t>Structured total</t>
+  </si>
+  <si>
+    <t>Named input</t>
+  </si>
+  <si>
+    <t>Indirect ref</t>
+  </si>
+  <si>
+    <t>Offset ref</t>
+  </si>
+  <si>
+    <t>External value</t>
   </si>
   <si>
     <t>Tax model</t>
@@ -143,6 +161,19 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpexTable" displayName="OpexTable" ref="A1:D6" totalsRowShown="0">
+  <autoFilter ref="A1:D6"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Item"/>
+    <tableColumn id="2" name="Amount"/>
+    <tableColumn id="3" name="Inflated"/>
+    <tableColumn id="4" name="Multiplier"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -562,12 +593,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -647,6 +681,51 @@
       </c>
       <c r="B9">
         <f>1+1</f>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10">
+        <f>SUM(OpexTable[Amount])</f>
+        <v>660</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <f>RevenueInput*2</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12">
+        <f>INDIRECT("Inputs!B3")*1000</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13">
+        <f>OFFSET(Inputs!B2,1,0)</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14">
+        <f>[external_book.xlsx]Sheet1!A1</f>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -661,15 +740,15 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <f>D3*0.1</f>

</xml_diff>

<commit_message>
feat: slice minimality and independent recalculation evidence
</commit_message>
<xml_diff>
--- a/fixtures/bad_model.xlsx
+++ b/fixtures/bad_model.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="B3">
         <f>SUM(Opex!C2:C6)</f>
-        <v>660</v>
+        <v>539</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -689,7 +689,7 @@
       </c>
       <c r="B10">
         <f>SUM(OpexTable[Amount])</f>
-        <v>660</v>
+        <v>640</v>
       </c>
     </row>
     <row r="11" spans="1:2">

</xml_diff>